<commit_message>
İP5: Random Forest yerine baştan XGBoost kullanılacak şekilde temizlik
ip5-random-forest/ klasörü ip5-adaptif-akts/ olarak yeniden adlandırıldı
(içerik zaten XGBoost kullanıyordu, isim buna göre düzeltildi). Tüm kod,
notebook ve rapor referansları güncellendi. Pipeline ve notebooklar
yeniden çalıştırılıp doğrulandı.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/ip6-validasyon/bloom_duzeyi_sapma_ozet.xlsx
+++ b/ip6-validasyon/bloom_duzeyi_sapma_ozet.xlsx
@@ -446,10 +446,10 @@
         <v>2810</v>
       </c>
       <c r="C2" t="n">
-        <v>8.27</v>
+        <v>8.369999999999999</v>
       </c>
       <c r="D2" t="n">
-        <v>29.91</v>
+        <v>24.02</v>
       </c>
     </row>
     <row r="3">
@@ -460,10 +460,10 @@
         <v>579</v>
       </c>
       <c r="C3" t="n">
-        <v>8.99</v>
+        <v>9.1</v>
       </c>
       <c r="D3" t="n">
-        <v>23.76</v>
+        <v>21.28</v>
       </c>
     </row>
     <row r="4">
@@ -474,10 +474,10 @@
         <v>491</v>
       </c>
       <c r="C4" t="n">
-        <v>12.34</v>
+        <v>11.06</v>
       </c>
       <c r="D4" t="n">
-        <v>30.56</v>
+        <v>19.34</v>
       </c>
     </row>
     <row r="5">
@@ -488,10 +488,10 @@
         <v>112</v>
       </c>
       <c r="C5" t="n">
-        <v>10.32</v>
+        <v>11.96</v>
       </c>
       <c r="D5" t="n">
-        <v>18.83</v>
+        <v>22.75</v>
       </c>
     </row>
     <row r="6">
@@ -502,10 +502,10 @@
         <v>34</v>
       </c>
       <c r="C6" t="n">
-        <v>16.53</v>
+        <v>15.16</v>
       </c>
       <c r="D6" t="n">
-        <v>15.98</v>
+        <v>21.87</v>
       </c>
     </row>
     <row r="7">
@@ -516,10 +516,10 @@
         <v>107</v>
       </c>
       <c r="C7" t="n">
-        <v>22.52</v>
+        <v>20.1</v>
       </c>
       <c r="D7" t="n">
-        <v>40.71</v>
+        <v>38.12</v>
       </c>
     </row>
   </sheetData>

</xml_diff>